<commit_message>
Update footer links for migrated pages, import 2 missing pages
Footer navigation:
- Newsroom: changed from absolute hp.com URL to relative /newsroom
- Contact HP: /contact-hp/overview (stripped .html)
- HP Partner Programs: /hp-information/partners-and-programs (relative)
- Developers: /developers (relative)
- Recalls, Recycling, Accessibility, Privacy, Terms: all relative paths
- Your privacy choices: kept absolute (page now migrated)
- Shop/support links: kept absolute (correct by design)

Missing pages imported (55 total):
- /us-en/all-in-plan/laptops
- /us-en/privacy/your-privacy-choices

Redirects updated:
- /us-en/ and /us-en -> /us-en/home (homepage root)
- .html extensions for 2 new pages

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-product-marketing.report.xlsx
+++ b/tools/importer/reports/import-product-marketing.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="283">
   <si>
     <t>_reportFile</t>
   </si>
@@ -106,6 +106,21 @@
     <t>https://www.hp.com/us-en/desktops.html</t>
   </si>
   <si>
+    <t>us-en/developers.report.json</t>
+  </si>
+  <si>
+    <t>us-en/developers</t>
+  </si>
+  <si>
+    <t>content-editorial</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:18:37.295Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/developers.html</t>
+  </si>
+  <si>
     <t>us-en/home.report.json</t>
   </si>
   <si>
@@ -136,9 +151,6 @@
     <t>us-en/hp-information</t>
   </si>
   <si>
-    <t>content-editorial</t>
-  </si>
-  <si>
     <t>2026-04-08T12:29:21.774Z</t>
   </si>
   <si>
@@ -244,6 +256,18 @@
     <t>https://www.hp.com/us-en/terms-of-use.html</t>
   </si>
   <si>
+    <t>us-en/all-in-plan/laptops.report.json</t>
+  </si>
+  <si>
+    <t>us-en/all-in-plan/laptops</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:36:05.636Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/all-in-plan/laptops.html</t>
+  </si>
+  <si>
     <t>us-en/all-in-plan/printers.report.json</t>
   </si>
   <si>
@@ -286,6 +310,21 @@
     <t>https://www.hp.com/us-en/business-solutions/services-solutions.html</t>
   </si>
   <si>
+    <t>us-en/contact-hp/contact.report.json</t>
+  </si>
+  <si>
+    <t>us-en/contact-hp/contact</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:18:50.109Z</t>
+  </si>
+  <si>
+    <t>Contact HP | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/contact-hp/contact.html</t>
+  </si>
+  <si>
     <t>us-en/contact-hp/overview.report.json</t>
   </si>
   <si>
@@ -454,6 +493,24 @@
     <t>https://www.hp.com/us-en/printers/home-printers.html</t>
   </si>
   <si>
+    <t>us-en/printers/instant-ink.report.json</t>
+  </si>
+  <si>
+    <t>["cards","cards","cards","cards"]</t>
+  </si>
+  <si>
+    <t>us-en/printers/instant-ink</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:19:42.832Z</t>
+  </si>
+  <si>
+    <t>HP Instant Ink – Printer Ink Subscription | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/printers/instant-ink.html</t>
+  </si>
+  <si>
     <t>us-en/printers/smart-tank.report.json</t>
   </si>
   <si>
@@ -487,6 +544,21 @@
     <t>https://www.hp.com/us-en/privacy/privacy-central.html</t>
   </si>
   <si>
+    <t>us-en/privacy/your-privacy-choices.report.json</t>
+  </si>
+  <si>
+    <t>us-en/privacy/your-privacy-choices</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:36:16.949Z</t>
+  </si>
+  <si>
+    <t>Your Privacy Choices | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/privacy/your-privacy-choices.html</t>
+  </si>
+  <si>
     <t>us-en/software/microsoft-copilot-pcs-for-home.report.json</t>
   </si>
   <si>
@@ -502,6 +574,81 @@
     <t>https://www.hp.com/us-en/software/microsoft-copilot-pcs-for-home.html</t>
   </si>
   <si>
+    <t>us-en/solutions/learning-hub.report.json</t>
+  </si>
+  <si>
+    <t>us-en/solutions/learning-hub</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:19:16.749Z</t>
+  </si>
+  <si>
+    <t>HP Solutions Learning Hub | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/solutions/learning-hub.html</t>
+  </si>
+  <si>
+    <t>us-en/workstations/learning-hub.report.json</t>
+  </si>
+  <si>
+    <t>["hero","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards"]</t>
+  </si>
+  <si>
+    <t>us-en/workstations/learning-hub</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:19:05.817Z</t>
+  </si>
+  <si>
+    <t>Z Workstation Computers Whitepapers, Case Studies, and Resources | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/workstations/learning-hub.html</t>
+  </si>
+  <si>
+    <t>us-en/hp-information/about-hp/inclusion.report.json</t>
+  </si>
+  <si>
+    <t>["hero","cards","cards","cards","cards","cards"]</t>
+  </si>
+  <si>
+    <t>us-en/hp-information/about-hp/inclusion</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:18:03.589Z</t>
+  </si>
+  <si>
+    <t>Inclusion at HP | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/hp-information/about-hp/inclusion.html</t>
+  </si>
+  <si>
+    <t>us-en/hp-information/sustainable-impact/climate-action.report.json</t>
+  </si>
+  <si>
+    <t>us-en/hp-information/sustainable-impact/climate-action</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:18:13.958Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/hp-information/sustainable-impact/climate-action.html</t>
+  </si>
+  <si>
+    <t>us-en/hp-information/sustainable-impact/human-rights.report.json</t>
+  </si>
+  <si>
+    <t>us-en/hp-information/sustainable-impact/human-rights</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:18:25.865Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/hp-information/sustainable-impact/human-rights.html</t>
+  </si>
+  <si>
     <t>us-en/hp-information/sustainable-impact/planet-product-recycling.report.json</t>
   </si>
   <si>
@@ -517,6 +664,18 @@
     <t>https://www.hp.com/us-en/hp-information/sustainable-impact/planet-product-recycling.html</t>
   </si>
   <si>
+    <t>us-en/printers/smart-tank/smart-tank-benefits.report.json</t>
+  </si>
+  <si>
+    <t>us-en/printers/smart-tank/smart-tank-benefits</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:19:29.154Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/printers/smart-tank/smart-tank-benefits.html</t>
+  </si>
+  <si>
     <t>us-en/resources/case-study/work-from-space.report.json</t>
   </si>
   <si>
@@ -535,9 +694,6 @@
     <t>us-en/solutions/learning-hub/kinepolis-case-study.report.json</t>
   </si>
   <si>
-    <t>["hero","cards","cards","cards","cards","cards"]</t>
-  </si>
-  <si>
     <t>us-en/solutions/learning-hub/kinepolis-case-study</t>
   </si>
   <si>
@@ -586,6 +742,18 @@
     <t>https://www.hp.com/us-en/workstations/learning-hub/zaha-hadid-architects.html</t>
   </si>
   <si>
+    <t>us-en/newsroom/blogs/2025/hp-hybrid-work-trends.report.json</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/blogs/2025/hp-hybrid-work-trends</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:17:39.359Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/newsroom/blogs/2025/hp-hybrid-work-trends.html</t>
+  </si>
+  <si>
     <t>us-en/newsroom/blogs/2026/hp-2026-future-of-work-accelerator-selections.report.json</t>
   </si>
   <si>
@@ -601,6 +769,18 @@
     <t>https://www.hp.com/us-en/newsroom/blogs/2026/hp-2026-future-of-work-accelerator-selections.html</t>
   </si>
   <si>
+    <t>us-en/newsroom/press-releases/2024/hp-amplify-partner-program.report.json</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/press-releases/2024/hp-amplify-partner-program</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:17:50.854Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/newsroom/press-releases/2024/hp-amplify-partner-program.html</t>
+  </si>
+  <si>
     <t>us-en/newsroom/press-releases/2024/hp-wri-reveals-ai-unlock-better-work-relationships.report.json</t>
   </si>
   <si>
@@ -614,6 +794,42 @@
   </si>
   <si>
     <t>https://www.hp.com/us-en/newsroom/press-releases/2024/hp-wri-reveals-ai-unlock-better-work-relationships.html</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/press-releases/2025/hp-next-gen-ai-pcs.report.json</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/press-releases/2025/hp-next-gen-ai-pcs</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:17:08.451Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/newsroom/press-releases/2025/hp-next-gen-ai-pcs.html</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/press-releases/2025/hp-omnibook-ultra-launch.report.json</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/press-releases/2025/hp-omnibook-ultra-launch</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:17:16.016Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/newsroom/press-releases/2025/hp-omnibook-ultra-launch.html</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/press-releases/2025/hp-sustainability-report.report.json</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/press-releases/2025/hp-sustainability-report</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:17:27.200Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/newsroom/press-releases/2025/hp-sustainability-report.html</t>
   </si>
   <si>
     <t>us-en/newsroom/press-releases/2026/hp-pc-local-compute-ai-workloads.report.json</t>
@@ -1032,7 +1248,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -1176,88 +1392,88 @@
         <v>31</v>
       </c>
       <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
         <v>32</v>
       </c>
-      <c r="C6" t="s">
-        <v>33</v>
-      </c>
       <c r="D6" t="s">
         <v>11</v>
       </c>
       <c r="E6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" t="s">
         <v>34</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" t="s">
         <v>35</v>
-      </c>
-      <c r="G6" t="s">
-        <v>36</v>
-      </c>
-      <c r="H6" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" t="s">
         <v>38</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
         <v>39</v>
       </c>
-      <c r="C7" t="s">
+      <c r="F7" t="s">
         <v>40</v>
       </c>
-      <c r="D7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" t="s">
+      <c r="G7" t="s">
         <v>41</v>
       </c>
-      <c r="F7" t="s">
+      <c r="H7" t="s">
         <v>42</v>
-      </c>
-      <c r="G7" t="s">
-        <v>43</v>
-      </c>
-      <c r="H7" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" t="s">
         <v>45</v>
       </c>
-      <c r="B8" t="s">
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" t="s">
         <v>46</v>
       </c>
-      <c r="C8" t="s">
+      <c r="G8" t="s">
         <v>47</v>
       </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="H8" t="s">
         <v>48</v>
-      </c>
-      <c r="G8" t="s">
-        <v>49</v>
-      </c>
-      <c r="H8" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" t="s">
         <v>51</v>
-      </c>
-      <c r="B9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" t="s">
-        <v>52</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -1266,10 +1482,10 @@
         <v>12</v>
       </c>
       <c r="F9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" t="s">
         <v>53</v>
-      </c>
-      <c r="G9" t="s">
-        <v>14</v>
       </c>
       <c r="H9" t="s">
         <v>54</v>
@@ -1280,140 +1496,140 @@
         <v>55</v>
       </c>
       <c r="B10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
         <v>56</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" t="s">
         <v>57</v>
       </c>
-      <c r="D10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" t="s">
-        <v>41</v>
-      </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
+        <v>14</v>
+      </c>
+      <c r="H10" t="s">
         <v>58</v>
-      </c>
-      <c r="G10" t="s">
-        <v>59</v>
-      </c>
-      <c r="H10" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" t="s">
         <v>61</v>
       </c>
-      <c r="B11" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" t="s">
         <v>62</v>
       </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>63</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>64</v>
-      </c>
-      <c r="H11" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
         <v>66</v>
       </c>
-      <c r="B12" t="s">
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" t="s">
         <v>67</v>
       </c>
-      <c r="C12" t="s">
+      <c r="G12" t="s">
         <v>68</v>
       </c>
-      <c r="D12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" t="s">
-        <v>41</v>
-      </c>
-      <c r="F12" t="s">
+      <c r="H12" t="s">
         <v>69</v>
-      </c>
-      <c r="G12" t="s">
-        <v>70</v>
-      </c>
-      <c r="H12" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" t="s">
         <v>72</v>
       </c>
-      <c r="B13" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" t="s">
         <v>73</v>
       </c>
-      <c r="D13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" t="s">
-        <v>41</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>74</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>75</v>
-      </c>
-      <c r="H13" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>76</v>
+      </c>
+      <c r="B14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
         <v>77</v>
       </c>
-      <c r="B14" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>33</v>
+      </c>
+      <c r="F14" t="s">
         <v>78</v>
       </c>
-      <c r="D14" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" t="s">
-        <v>18</v>
-      </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>79</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>80</v>
-      </c>
-      <c r="H14" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>81</v>
+      </c>
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" t="s">
         <v>82</v>
-      </c>
-      <c r="B15" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15" t="s">
-        <v>83</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
@@ -1422,24 +1638,24 @@
         <v>18</v>
       </c>
       <c r="F15" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G15" t="s">
         <v>14</v>
       </c>
       <c r="H15" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>85</v>
+      </c>
+      <c r="B16" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" t="s">
         <v>86</v>
-      </c>
-      <c r="B16" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16" t="s">
-        <v>87</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
@@ -1448,50 +1664,50 @@
         <v>18</v>
       </c>
       <c r="F16" t="s">
+        <v>87</v>
+      </c>
+      <c r="G16" t="s">
         <v>88</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>89</v>
-      </c>
-      <c r="H16" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>90</v>
+      </c>
+      <c r="B17" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" t="s">
         <v>91</v>
       </c>
-      <c r="B17" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>18</v>
+      </c>
+      <c r="F17" t="s">
         <v>92</v>
-      </c>
-      <c r="D17" t="s">
-        <v>11</v>
-      </c>
-      <c r="E17" t="s">
-        <v>41</v>
-      </c>
-      <c r="F17" t="s">
-        <v>93</v>
       </c>
       <c r="G17" t="s">
         <v>14</v>
       </c>
       <c r="H17" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>94</v>
+      </c>
+      <c r="B18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" t="s">
         <v>95</v>
-      </c>
-      <c r="B18" t="s">
-        <v>9</v>
-      </c>
-      <c r="C18" t="s">
-        <v>96</v>
       </c>
       <c r="D18" t="s">
         <v>11</v>
@@ -1500,10 +1716,10 @@
         <v>18</v>
       </c>
       <c r="F18" t="s">
+        <v>96</v>
+      </c>
+      <c r="G18" t="s">
         <v>97</v>
-      </c>
-      <c r="G18" t="s">
-        <v>14</v>
       </c>
       <c r="H18" t="s">
         <v>98</v>
@@ -1523,65 +1739,65 @@
         <v>11</v>
       </c>
       <c r="E19" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="F19" t="s">
         <v>101</v>
       </c>
       <c r="G19" t="s">
-        <v>14</v>
+        <v>102</v>
       </c>
       <c r="H19" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B20" t="s">
         <v>9</v>
       </c>
       <c r="C20" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D20" t="s">
         <v>11</v>
       </c>
       <c r="E20" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="F20" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G20" t="s">
         <v>14</v>
       </c>
       <c r="H20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B21" t="s">
         <v>9</v>
       </c>
       <c r="C21" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D21" t="s">
         <v>11</v>
       </c>
       <c r="E21" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="F21" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G21" t="s">
-        <v>110</v>
+        <v>14</v>
       </c>
       <c r="H21" t="s">
         <v>111</v>
@@ -1592,166 +1808,166 @@
         <v>112</v>
       </c>
       <c r="B22" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" t="s">
         <v>113</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" t="s">
+        <v>18</v>
+      </c>
+      <c r="F22" t="s">
         <v>114</v>
       </c>
-      <c r="D22" t="s">
-        <v>11</v>
-      </c>
-      <c r="E22" t="s">
-        <v>41</v>
-      </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
+        <v>14</v>
+      </c>
+      <c r="H22" t="s">
         <v>115</v>
-      </c>
-      <c r="G22" t="s">
-        <v>116</v>
-      </c>
-      <c r="H22" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>116</v>
+      </c>
+      <c r="B23" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" t="s">
+        <v>117</v>
+      </c>
+      <c r="D23" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" t="s">
+        <v>18</v>
+      </c>
+      <c r="F23" t="s">
         <v>118</v>
-      </c>
-      <c r="B23" t="s">
-        <v>9</v>
-      </c>
-      <c r="C23" t="s">
-        <v>119</v>
-      </c>
-      <c r="D23" t="s">
-        <v>11</v>
-      </c>
-      <c r="E23" t="s">
-        <v>41</v>
-      </c>
-      <c r="F23" t="s">
-        <v>120</v>
       </c>
       <c r="G23" t="s">
         <v>14</v>
       </c>
       <c r="H23" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>120</v>
+      </c>
+      <c r="B24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" t="s">
+        <v>121</v>
+      </c>
+      <c r="D24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" t="s">
+        <v>33</v>
+      </c>
+      <c r="F24" t="s">
         <v>122</v>
       </c>
-      <c r="B24" t="s">
-        <v>9</v>
-      </c>
-      <c r="C24" t="s">
+      <c r="G24" t="s">
         <v>123</v>
       </c>
-      <c r="D24" t="s">
-        <v>11</v>
-      </c>
-      <c r="E24" t="s">
-        <v>41</v>
-      </c>
-      <c r="F24" t="s">
+      <c r="H24" t="s">
         <v>124</v>
-      </c>
-      <c r="G24" t="s">
-        <v>125</v>
-      </c>
-      <c r="H24" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>125</v>
+      </c>
+      <c r="B25" t="s">
+        <v>126</v>
+      </c>
+      <c r="C25" t="s">
         <v>127</v>
       </c>
-      <c r="B25" t="s">
-        <v>9</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" t="s">
+        <v>33</v>
+      </c>
+      <c r="F25" t="s">
         <v>128</v>
       </c>
-      <c r="D25" t="s">
-        <v>11</v>
-      </c>
-      <c r="E25" t="s">
-        <v>18</v>
-      </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
         <v>129</v>
       </c>
-      <c r="G25" t="s">
+      <c r="H25" t="s">
         <v>130</v>
-      </c>
-      <c r="H25" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" t="s">
+        <v>9</v>
+      </c>
+      <c r="C26" t="s">
         <v>132</v>
       </c>
-      <c r="B26" t="s">
-        <v>9</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" t="s">
+        <v>33</v>
+      </c>
+      <c r="F26" t="s">
         <v>133</v>
       </c>
-      <c r="D26" t="s">
-        <v>11</v>
-      </c>
-      <c r="E26" t="s">
-        <v>18</v>
-      </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
+        <v>14</v>
+      </c>
+      <c r="H26" t="s">
         <v>134</v>
-      </c>
-      <c r="G26" t="s">
-        <v>135</v>
-      </c>
-      <c r="H26" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>135</v>
+      </c>
+      <c r="B27" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" t="s">
+        <v>136</v>
+      </c>
+      <c r="D27" t="s">
+        <v>11</v>
+      </c>
+      <c r="E27" t="s">
+        <v>33</v>
+      </c>
+      <c r="F27" t="s">
         <v>137</v>
       </c>
-      <c r="B27" t="s">
-        <v>9</v>
-      </c>
-      <c r="C27" t="s">
+      <c r="G27" t="s">
         <v>138</v>
       </c>
-      <c r="D27" t="s">
-        <v>11</v>
-      </c>
-      <c r="E27" t="s">
-        <v>18</v>
-      </c>
-      <c r="F27" t="s">
+      <c r="H27" t="s">
         <v>139</v>
-      </c>
-      <c r="G27" t="s">
-        <v>140</v>
-      </c>
-      <c r="H27" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B28" t="s">
         <v>9</v>
       </c>
       <c r="C28" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D28" t="s">
         <v>11</v>
@@ -1760,24 +1976,24 @@
         <v>18</v>
       </c>
       <c r="F28" t="s">
+        <v>142</v>
+      </c>
+      <c r="G28" t="s">
+        <v>143</v>
+      </c>
+      <c r="H28" t="s">
         <v>144</v>
-      </c>
-      <c r="G28" t="s">
-        <v>145</v>
-      </c>
-      <c r="H28" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B29" t="s">
-        <v>148</v>
+        <v>9</v>
       </c>
       <c r="C29" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D29" t="s">
         <v>11</v>
@@ -1786,50 +2002,50 @@
         <v>18</v>
       </c>
       <c r="F29" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="G29" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H29" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>150</v>
+      </c>
+      <c r="B30" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" t="s">
+        <v>151</v>
+      </c>
+      <c r="D30" t="s">
+        <v>11</v>
+      </c>
+      <c r="E30" t="s">
+        <v>18</v>
+      </c>
+      <c r="F30" t="s">
+        <v>152</v>
+      </c>
+      <c r="G30" t="s">
         <v>153</v>
       </c>
-      <c r="B30" t="s">
-        <v>39</v>
-      </c>
-      <c r="C30" t="s">
+      <c r="H30" t="s">
         <v>154</v>
-      </c>
-      <c r="D30" t="s">
-        <v>11</v>
-      </c>
-      <c r="E30" t="s">
-        <v>41</v>
-      </c>
-      <c r="F30" t="s">
-        <v>155</v>
-      </c>
-      <c r="G30" t="s">
-        <v>156</v>
-      </c>
-      <c r="H30" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B31" t="s">
         <v>9</v>
       </c>
       <c r="C31" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D31" t="s">
         <v>11</v>
@@ -1838,247 +2054,663 @@
         <v>18</v>
       </c>
       <c r="F31" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G31" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H31" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>160</v>
+      </c>
+      <c r="B32" t="s">
+        <v>161</v>
+      </c>
+      <c r="C32" t="s">
+        <v>162</v>
+      </c>
+      <c r="D32" t="s">
+        <v>11</v>
+      </c>
+      <c r="E32" t="s">
+        <v>33</v>
+      </c>
+      <c r="F32" t="s">
         <v>163</v>
       </c>
-      <c r="B32" t="s">
-        <v>113</v>
-      </c>
-      <c r="C32" t="s">
+      <c r="G32" t="s">
         <v>164</v>
       </c>
-      <c r="D32" t="s">
-        <v>11</v>
-      </c>
-      <c r="E32" t="s">
-        <v>41</v>
-      </c>
-      <c r="F32" t="s">
+      <c r="H32" t="s">
         <v>165</v>
-      </c>
-      <c r="G32" t="s">
-        <v>166</v>
-      </c>
-      <c r="H32" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>166</v>
+      </c>
+      <c r="B33" t="s">
+        <v>167</v>
+      </c>
+      <c r="C33" t="s">
         <v>168</v>
       </c>
-      <c r="B33" t="s">
-        <v>9</v>
-      </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
+        <v>11</v>
+      </c>
+      <c r="E33" t="s">
+        <v>18</v>
+      </c>
+      <c r="F33" t="s">
         <v>169</v>
       </c>
-      <c r="D33" t="s">
-        <v>11</v>
-      </c>
-      <c r="E33" t="s">
-        <v>41</v>
-      </c>
-      <c r="F33" t="s">
+      <c r="G33" t="s">
         <v>170</v>
       </c>
-      <c r="G33" t="s">
+      <c r="H33" t="s">
         <v>171</v>
-      </c>
-      <c r="H33" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>172</v>
+      </c>
+      <c r="B34" t="s">
+        <v>44</v>
+      </c>
+      <c r="C34" t="s">
         <v>173</v>
       </c>
-      <c r="B34" t="s">
+      <c r="D34" t="s">
+        <v>11</v>
+      </c>
+      <c r="E34" t="s">
+        <v>33</v>
+      </c>
+      <c r="F34" t="s">
         <v>174</v>
       </c>
-      <c r="C34" t="s">
+      <c r="G34" t="s">
         <v>175</v>
       </c>
-      <c r="D34" t="s">
-        <v>11</v>
-      </c>
-      <c r="E34" t="s">
-        <v>41</v>
-      </c>
-      <c r="F34" t="s">
+      <c r="H34" t="s">
         <v>176</v>
-      </c>
-      <c r="G34" t="s">
-        <v>177</v>
-      </c>
-      <c r="H34" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>177</v>
+      </c>
+      <c r="B35" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" t="s">
+        <v>178</v>
+      </c>
+      <c r="D35" t="s">
+        <v>11</v>
+      </c>
+      <c r="E35" t="s">
+        <v>18</v>
+      </c>
+      <c r="F35" t="s">
         <v>179</v>
       </c>
-      <c r="B35" t="s">
+      <c r="G35" t="s">
         <v>180</v>
       </c>
-      <c r="C35" t="s">
+      <c r="H35" t="s">
         <v>181</v>
-      </c>
-      <c r="D35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E35" t="s">
-        <v>41</v>
-      </c>
-      <c r="F35" t="s">
-        <v>182</v>
-      </c>
-      <c r="G35" t="s">
-        <v>183</v>
-      </c>
-      <c r="H35" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>182</v>
+      </c>
+      <c r="B36" t="s">
+        <v>9</v>
+      </c>
+      <c r="C36" t="s">
+        <v>183</v>
+      </c>
+      <c r="D36" t="s">
+        <v>11</v>
+      </c>
+      <c r="E36" t="s">
+        <v>18</v>
+      </c>
+      <c r="F36" t="s">
+        <v>184</v>
+      </c>
+      <c r="G36" t="s">
         <v>185</v>
       </c>
-      <c r="B36" t="s">
+      <c r="H36" t="s">
         <v>186</v>
-      </c>
-      <c r="C36" t="s">
-        <v>187</v>
-      </c>
-      <c r="D36" t="s">
-        <v>11</v>
-      </c>
-      <c r="E36" t="s">
-        <v>41</v>
-      </c>
-      <c r="F36" t="s">
-        <v>188</v>
-      </c>
-      <c r="G36" t="s">
-        <v>189</v>
-      </c>
-      <c r="H36" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>187</v>
+      </c>
+      <c r="B37" t="s">
+        <v>60</v>
+      </c>
+      <c r="C37" t="s">
+        <v>188</v>
+      </c>
+      <c r="D37" t="s">
+        <v>11</v>
+      </c>
+      <c r="E37" t="s">
+        <v>33</v>
+      </c>
+      <c r="F37" t="s">
+        <v>189</v>
+      </c>
+      <c r="G37" t="s">
+        <v>190</v>
+      </c>
+      <c r="H37" t="s">
         <v>191</v>
-      </c>
-      <c r="B37" t="s">
-        <v>174</v>
-      </c>
-      <c r="C37" t="s">
-        <v>192</v>
-      </c>
-      <c r="D37" t="s">
-        <v>11</v>
-      </c>
-      <c r="E37" t="s">
-        <v>41</v>
-      </c>
-      <c r="F37" t="s">
-        <v>193</v>
-      </c>
-      <c r="G37" t="s">
-        <v>194</v>
-      </c>
-      <c r="H37" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>192</v>
+      </c>
+      <c r="B38" t="s">
+        <v>193</v>
+      </c>
+      <c r="C38" t="s">
+        <v>194</v>
+      </c>
+      <c r="D38" t="s">
+        <v>11</v>
+      </c>
+      <c r="E38" t="s">
+        <v>33</v>
+      </c>
+      <c r="F38" t="s">
+        <v>195</v>
+      </c>
+      <c r="G38" t="s">
         <v>196</v>
       </c>
-      <c r="B38" t="s">
-        <v>174</v>
-      </c>
-      <c r="C38" t="s">
+      <c r="H38" t="s">
         <v>197</v>
-      </c>
-      <c r="D38" t="s">
-        <v>11</v>
-      </c>
-      <c r="E38" t="s">
-        <v>41</v>
-      </c>
-      <c r="F38" t="s">
-        <v>198</v>
-      </c>
-      <c r="G38" t="s">
-        <v>199</v>
-      </c>
-      <c r="H38" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>198</v>
+      </c>
+      <c r="B39" t="s">
+        <v>199</v>
+      </c>
+      <c r="C39" t="s">
+        <v>200</v>
+      </c>
+      <c r="D39" t="s">
+        <v>11</v>
+      </c>
+      <c r="E39" t="s">
+        <v>33</v>
+      </c>
+      <c r="F39" t="s">
         <v>201</v>
       </c>
-      <c r="B39" t="s">
-        <v>174</v>
-      </c>
-      <c r="C39" t="s">
+      <c r="G39" t="s">
         <v>202</v>
       </c>
-      <c r="D39" t="s">
-        <v>11</v>
-      </c>
-      <c r="E39" t="s">
-        <v>41</v>
-      </c>
-      <c r="F39" t="s">
+      <c r="H39" t="s">
         <v>203</v>
-      </c>
-      <c r="G39" t="s">
-        <v>204</v>
-      </c>
-      <c r="H39" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>204</v>
+      </c>
+      <c r="B40" t="s">
+        <v>9</v>
+      </c>
+      <c r="C40" t="s">
+        <v>205</v>
+      </c>
+      <c r="D40" t="s">
+        <v>11</v>
+      </c>
+      <c r="E40" t="s">
+        <v>33</v>
+      </c>
+      <c r="F40" t="s">
         <v>206</v>
       </c>
-      <c r="B40" t="s">
-        <v>174</v>
-      </c>
-      <c r="C40" t="s">
+      <c r="G40" t="s">
+        <v>14</v>
+      </c>
+      <c r="H40" t="s">
         <v>207</v>
       </c>
-      <c r="D40" t="s">
-        <v>11</v>
-      </c>
-      <c r="E40" t="s">
-        <v>41</v>
-      </c>
-      <c r="F40" t="s">
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>208</v>
       </c>
-      <c r="G40" t="s">
+      <c r="B41" t="s">
+        <v>9</v>
+      </c>
+      <c r="C41" t="s">
         <v>209</v>
       </c>
-      <c r="H40" t="s">
+      <c r="D41" t="s">
+        <v>11</v>
+      </c>
+      <c r="E41" t="s">
+        <v>33</v>
+      </c>
+      <c r="F41" t="s">
         <v>210</v>
+      </c>
+      <c r="G41" t="s">
+        <v>14</v>
+      </c>
+      <c r="H41" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>212</v>
+      </c>
+      <c r="B42" t="s">
+        <v>126</v>
+      </c>
+      <c r="C42" t="s">
+        <v>213</v>
+      </c>
+      <c r="D42" t="s">
+        <v>11</v>
+      </c>
+      <c r="E42" t="s">
+        <v>33</v>
+      </c>
+      <c r="F42" t="s">
+        <v>214</v>
+      </c>
+      <c r="G42" t="s">
+        <v>215</v>
+      </c>
+      <c r="H42" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>217</v>
+      </c>
+      <c r="B43" t="s">
+        <v>9</v>
+      </c>
+      <c r="C43" t="s">
+        <v>218</v>
+      </c>
+      <c r="D43" t="s">
+        <v>11</v>
+      </c>
+      <c r="E43" t="s">
+        <v>33</v>
+      </c>
+      <c r="F43" t="s">
+        <v>219</v>
+      </c>
+      <c r="G43" t="s">
+        <v>14</v>
+      </c>
+      <c r="H43" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>221</v>
+      </c>
+      <c r="B44" t="s">
+        <v>9</v>
+      </c>
+      <c r="C44" t="s">
+        <v>222</v>
+      </c>
+      <c r="D44" t="s">
+        <v>11</v>
+      </c>
+      <c r="E44" t="s">
+        <v>33</v>
+      </c>
+      <c r="F44" t="s">
+        <v>223</v>
+      </c>
+      <c r="G44" t="s">
+        <v>224</v>
+      </c>
+      <c r="H44" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>226</v>
+      </c>
+      <c r="B45" t="s">
+        <v>199</v>
+      </c>
+      <c r="C45" t="s">
+        <v>227</v>
+      </c>
+      <c r="D45" t="s">
+        <v>11</v>
+      </c>
+      <c r="E45" t="s">
+        <v>33</v>
+      </c>
+      <c r="F45" t="s">
+        <v>228</v>
+      </c>
+      <c r="G45" t="s">
+        <v>229</v>
+      </c>
+      <c r="H45" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>231</v>
+      </c>
+      <c r="B46" t="s">
+        <v>232</v>
+      </c>
+      <c r="C46" t="s">
+        <v>233</v>
+      </c>
+      <c r="D46" t="s">
+        <v>11</v>
+      </c>
+      <c r="E46" t="s">
+        <v>33</v>
+      </c>
+      <c r="F46" t="s">
+        <v>234</v>
+      </c>
+      <c r="G46" t="s">
+        <v>235</v>
+      </c>
+      <c r="H46" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>237</v>
+      </c>
+      <c r="B47" t="s">
+        <v>238</v>
+      </c>
+      <c r="C47" t="s">
+        <v>239</v>
+      </c>
+      <c r="D47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" t="s">
+        <v>33</v>
+      </c>
+      <c r="F47" t="s">
+        <v>240</v>
+      </c>
+      <c r="G47" t="s">
+        <v>241</v>
+      </c>
+      <c r="H47" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>243</v>
+      </c>
+      <c r="B48" t="s">
+        <v>9</v>
+      </c>
+      <c r="C48" t="s">
+        <v>244</v>
+      </c>
+      <c r="D48" t="s">
+        <v>11</v>
+      </c>
+      <c r="E48" t="s">
+        <v>33</v>
+      </c>
+      <c r="F48" t="s">
+        <v>245</v>
+      </c>
+      <c r="G48" t="s">
+        <v>14</v>
+      </c>
+      <c r="H48" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>247</v>
+      </c>
+      <c r="B49" t="s">
+        <v>199</v>
+      </c>
+      <c r="C49" t="s">
+        <v>248</v>
+      </c>
+      <c r="D49" t="s">
+        <v>11</v>
+      </c>
+      <c r="E49" t="s">
+        <v>33</v>
+      </c>
+      <c r="F49" t="s">
+        <v>249</v>
+      </c>
+      <c r="G49" t="s">
+        <v>250</v>
+      </c>
+      <c r="H49" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>252</v>
+      </c>
+      <c r="B50" t="s">
+        <v>9</v>
+      </c>
+      <c r="C50" t="s">
+        <v>253</v>
+      </c>
+      <c r="D50" t="s">
+        <v>11</v>
+      </c>
+      <c r="E50" t="s">
+        <v>33</v>
+      </c>
+      <c r="F50" t="s">
+        <v>254</v>
+      </c>
+      <c r="G50" t="s">
+        <v>14</v>
+      </c>
+      <c r="H50" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>256</v>
+      </c>
+      <c r="B51" t="s">
+        <v>199</v>
+      </c>
+      <c r="C51" t="s">
+        <v>257</v>
+      </c>
+      <c r="D51" t="s">
+        <v>11</v>
+      </c>
+      <c r="E51" t="s">
+        <v>33</v>
+      </c>
+      <c r="F51" t="s">
+        <v>258</v>
+      </c>
+      <c r="G51" t="s">
+        <v>259</v>
+      </c>
+      <c r="H51" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>261</v>
+      </c>
+      <c r="B52" t="s">
+        <v>9</v>
+      </c>
+      <c r="C52" t="s">
+        <v>262</v>
+      </c>
+      <c r="D52" t="s">
+        <v>11</v>
+      </c>
+      <c r="E52" t="s">
+        <v>33</v>
+      </c>
+      <c r="F52" t="s">
+        <v>263</v>
+      </c>
+      <c r="G52" t="s">
+        <v>14</v>
+      </c>
+      <c r="H52" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>265</v>
+      </c>
+      <c r="B53" t="s">
+        <v>9</v>
+      </c>
+      <c r="C53" t="s">
+        <v>266</v>
+      </c>
+      <c r="D53" t="s">
+        <v>11</v>
+      </c>
+      <c r="E53" t="s">
+        <v>33</v>
+      </c>
+      <c r="F53" t="s">
+        <v>267</v>
+      </c>
+      <c r="G53" t="s">
+        <v>14</v>
+      </c>
+      <c r="H53" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>269</v>
+      </c>
+      <c r="B54" t="s">
+        <v>9</v>
+      </c>
+      <c r="C54" t="s">
+        <v>270</v>
+      </c>
+      <c r="D54" t="s">
+        <v>11</v>
+      </c>
+      <c r="E54" t="s">
+        <v>33</v>
+      </c>
+      <c r="F54" t="s">
+        <v>271</v>
+      </c>
+      <c r="G54" t="s">
+        <v>14</v>
+      </c>
+      <c r="H54" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>273</v>
+      </c>
+      <c r="B55" t="s">
+        <v>199</v>
+      </c>
+      <c r="C55" t="s">
+        <v>274</v>
+      </c>
+      <c r="D55" t="s">
+        <v>11</v>
+      </c>
+      <c r="E55" t="s">
+        <v>33</v>
+      </c>
+      <c r="F55" t="s">
+        <v>275</v>
+      </c>
+      <c r="G55" t="s">
+        <v>276</v>
+      </c>
+      <c r="H55" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>278</v>
+      </c>
+      <c r="B56" t="s">
+        <v>199</v>
+      </c>
+      <c r="C56" t="s">
+        <v>279</v>
+      </c>
+      <c r="D56" t="s">
+        <v>11</v>
+      </c>
+      <c r="E56" t="s">
+        <v>33</v>
+      </c>
+      <c r="F56" t="s">
+        <v>280</v>
+      </c>
+      <c r="G56" t="s">
+        <v>281</v>
+      </c>
+      <c r="H56" t="s">
+        <v>282</v>
       </c>
     </row>
   </sheetData>

</xml_diff>